<commit_message>
Regenerate the migration workbook and update chart tests for payroll accounts
The chart template now carries the approved payroll accounts 1230, 1240, 2330,
2340 and 5120, so the generated migration workbook and the monetary-account
lists of the FX tests change with it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVy7Y2kCiQ1NrNgFBo2Zhn
</commit_message>
<xml_diff>
--- a/docs/migration/almiras-migration-workbook.xlsx
+++ b/docs/migration/almiras-migration-workbook.xlsx
@@ -44,7 +44,7 @@
     <definedName name="L_checklist_status">'Lists'!$R$2:$R$4</definedName>
     <definedName name="L_currency">'Lists'!$S$2:$S$18</definedName>
     <definedName name="L_country">'Lists'!$T$2:$T$250</definedName>
-    <definedName name="L_erp_code">'Lists'!$U$2:$U$64</definedName>
+    <definedName name="L_erp_code">'Lists'!$U$2:$U$69</definedName>
     <definedName name="L_entity">'Entities'!$A$6:$A$2005</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3179,7 +3179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3587,17 +3587,17 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>1300</t>
+          <t>1230</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sharia-compliant deposits (e.g. murabaha, wakala)</t>
+          <t>Employee loans and advances</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>ودائع متوافقة مع الشريعة</t>
+          <t>قروض وسلف الموظفين</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -3629,17 +3629,17 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>1310</t>
+          <t>1240</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>VAT input</t>
+          <t>Employee deferred-sale (bai' ajel) receivable</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>ضريبة القيمة المضافة - مدخلات</t>
+          <t>ذمم البيع الآجل للموظفين</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -3671,17 +3671,17 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>1320</t>
+          <t>1300</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Prepayments</t>
+          <t>Sharia-compliant deposits (e.g. murabaha, wakala)</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>مصروفات مدفوعة مقدماً</t>
+          <t>ودائع متوافقة مع الشريعة</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -3713,17 +3713,17 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>1400</t>
+          <t>1310</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Investments in subsidiaries</t>
+          <t>VAT input</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>استثمارات في شركات تابعة</t>
+          <t>ضريبة القيمة المضافة - مدخلات</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -3755,17 +3755,17 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>1410</t>
+          <t>1320</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Investments in associates (equity method)</t>
+          <t>Prepayments</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>استثمارات في شركات زميلة</t>
+          <t>مصروفات مدفوعة مقدماً</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -3797,17 +3797,17 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>1420</t>
+          <t>1400</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Other equity investments</t>
+          <t>Investments in subsidiaries</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>استثمارات حقوق ملكية أخرى</t>
+          <t>استثمارات في شركات تابعة</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -3839,17 +3839,17 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>1410</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Property, plant and equipment</t>
+          <t>Investments in associates (equity method)</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>الممتلكات والآلات والمعدات</t>
+          <t>استثمارات في شركات زميلة</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -3881,17 +3881,17 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>1510</t>
+          <t>1420</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Investment property (rental assets)</t>
+          <t>Other equity investments</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>عقارات استثمارية</t>
+          <t>استثمارات حقوق ملكية أخرى</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -3923,17 +3923,17 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>1520</t>
+          <t>1500</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Vehicles</t>
+          <t>Property, plant and equipment</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>السيارات</t>
+          <t>الممتلكات والآلات والمعدات</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -3965,17 +3965,17 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>1590</t>
+          <t>1510</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Accumulated depreciation</t>
+          <t>Investment property (rental assets)</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>مجمع الاستهلاك</t>
+          <t>عقارات استثمارية</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -4007,17 +4007,17 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>1520</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Intangible assets and IP</t>
+          <t>Vehicles</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>الأصول غير الملموسة والملكية الفكرية</t>
+          <t>السيارات</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -4049,27 +4049,27 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>1590</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Liabilities</t>
+          <t>Accumulated depreciation</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>الالتزامات</t>
+          <t>مجمع الاستهلاك</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>liability</t>
+          <t>asset</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -4091,22 +4091,22 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>2100</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Trade payables</t>
+          <t>Intangible assets and IP</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>الذمم الدائنة التجارية</t>
+          <t>الأصول غير الملموسة والملكية الفكرية</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>liability</t>
+          <t>asset</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -4126,24 +4126,24 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Due to group entities</t>
+          <t>Liabilities</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>مستحق لشركات المجموعة</t>
+          <t>الالتزامات</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -4153,12 +4153,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -4168,24 +4168,24 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>2100</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>VAT output</t>
+          <t>Trade payables</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>ضريبة القيمة المضافة - مخرجات</t>
+          <t>الذمم الدائنة التجارية</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -4210,24 +4210,24 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>2210</t>
+          <t>2110</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Zakat payable</t>
+          <t>Due to group entities</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>الزكاة المستحقة</t>
+          <t>مستحق لشركات المجموعة</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -4242,7 +4242,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -4252,24 +4252,24 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>2220</t>
+          <t>2200</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Withholding tax payable</t>
+          <t>VAT output</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>ضريبة الاستقطاع المستحقة</t>
+          <t>ضريبة القيمة المضافة - مخرجات</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -4301,17 +4301,17 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>2300</t>
+          <t>2210</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Accrued expenses</t>
+          <t>Zakat payable</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>مصروفات مستحقة</t>
+          <t>الزكاة المستحقة</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -4343,17 +4343,17 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>2400</t>
+          <t>2220</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Islamic financing (murabaha, tawarruq)</t>
+          <t>Withholding tax payable</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>تمويل إسلامي</t>
+          <t>ضريبة الاستقطاع المستحقة</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -4385,17 +4385,17 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>2410</t>
+          <t>2300</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Conventional interest-bearing loans</t>
+          <t>Accrued expenses</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>قروض تقليدية بفائدة</t>
+          <t>مصروفات مستحقة</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -4415,7 +4415,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -4427,17 +4427,17 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>2500</t>
+          <t>2330</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>End-of-service provision</t>
+          <t>Salaries payable</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>مخصص مكافأة نهاية الخدمة</t>
+          <t>رواتب مستحقة</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -4469,17 +4469,17 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>2600</t>
+          <t>2340</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Charity payable (purification)</t>
+          <t>GOSI payable</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>مبالغ مستحقة للتطهير</t>
+          <t>اشتراكات التأمينات الاجتماعية المستحقة</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4511,27 +4511,27 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>3000</t>
+          <t>2400</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>Islamic financing (murabaha, tawarruq)</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>حقوق الملكية</t>
+          <t>تمويل إسلامي</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>equity</t>
+          <t>liability</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4553,22 +4553,22 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>3100</t>
+          <t>2410</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Share capital</t>
+          <t>Conventional interest-bearing loans</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>رأس المال</t>
+          <t>قروض تقليدية بفائدة</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>equity</t>
+          <t>liability</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -4595,22 +4595,22 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>3200</t>
+          <t>2500</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Statutory reserve</t>
+          <t>End-of-service provision</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>الاحتياطي النظامي</t>
+          <t>مخصص مكافأة نهاية الخدمة</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>equity</t>
+          <t>liability</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -4637,22 +4637,22 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>3300</t>
+          <t>2600</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Retained earnings</t>
+          <t>Charity payable (purification)</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>الأرباح المبقاة</t>
+          <t>مبالغ مستحقة للتطهير</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>equity</t>
+          <t>liability</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -4679,17 +4679,17 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>3400</t>
+          <t>3000</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Foreign currency translation reserve</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>احتياطي ترجمة العملات الأجنبية</t>
+          <t>حقوق الملكية</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4721,17 +4721,17 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>3900</t>
+          <t>3100</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Opening balance equity (migration)</t>
+          <t>Share capital</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>حقوق ملكية الأرصدة الافتتاحية</t>
+          <t>رأس المال</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -4763,27 +4763,27 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>4000</t>
+          <t>3200</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Statutory reserve</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>الإيرادات</t>
+          <t>الاحتياطي النظامي</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>income</t>
+          <t>equity</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4805,22 +4805,22 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>4100</t>
+          <t>3300</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Rental income</t>
+          <t>Retained earnings</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>إيرادات الإيجار</t>
+          <t>الأرباح المبقاة</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>income</t>
+          <t>equity</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -4847,27 +4847,27 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>4110</t>
+          <t>3400</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Intercompany rental income</t>
+          <t>Foreign currency translation reserve</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>إيرادات إيجار من شركات المجموعة</t>
+          <t>احتياطي ترجمة العملات الأجنبية</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>income</t>
+          <t>equity</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -4889,22 +4889,22 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>4120</t>
+          <t>3900</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Residential rental income (VAT-exempt)</t>
+          <t>Opening balance equity (migration)</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>إيرادات الإيجار السكني (معفاة)</t>
+          <t>حقوق ملكية الأرصدة الافتتاحية</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>income</t>
+          <t>equity</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -4931,17 +4931,17 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>4200</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Secondment and consulting income</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>إيرادات الإعارة والاستشارات</t>
+          <t>الإيرادات</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4951,7 +4951,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -4973,17 +4973,17 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>4210</t>
+          <t>4100</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Intercompany service income</t>
+          <t>Rental income</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>إيرادات خدمات من شركات المجموعة</t>
+          <t>إيرادات الإيجار</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -5015,17 +5015,17 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>4220</t>
+          <t>4110</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Management fee income</t>
+          <t>Intercompany rental income</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>إيرادات رسوم الإدارة</t>
+          <t>إيرادات إيجار من شركات المجموعة</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -5057,17 +5057,17 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>4230</t>
+          <t>4120</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Service charge income</t>
+          <t>Residential rental income (VAT-exempt)</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>إيرادات رسوم الخدمات المشتركة</t>
+          <t>إيرادات الإيجار السكني (معفاة)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5099,17 +5099,17 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>4240</t>
+          <t>4200</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Service fee income</t>
+          <t>Secondment and consulting income</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>إيرادات أتعاب الخدمات</t>
+          <t>إيرادات الإعارة والاستشارات</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5141,17 +5141,17 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>4300</t>
+          <t>4210</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>IP and licence income</t>
+          <t>Intercompany service income</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>إيرادات الملكية الفكرية والتراخيص</t>
+          <t>إيرادات خدمات من شركات المجموعة</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5183,17 +5183,17 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>4310</t>
+          <t>4220</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Intercompany IP and licence income</t>
+          <t>Management fee income</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>إيرادات ملكية فكرية من شركات المجموعة</t>
+          <t>إيرادات رسوم الإدارة</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -5225,17 +5225,17 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>4400</t>
+          <t>4230</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Dividend income</t>
+          <t>Service charge income</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>إيرادات توزيعات الأرباح</t>
+          <t>إيرادات رسوم الخدمات المشتركة</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -5267,17 +5267,17 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>4500</t>
+          <t>4240</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Share of profit of associates</t>
+          <t>Service fee income</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>الحصة من أرباح الشركات الزميلة</t>
+          <t>إيرادات أتعاب الخدمات</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -5309,17 +5309,17 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>4600</t>
+          <t>4300</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Islamic deposit profit</t>
+          <t>IP and licence income</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>أرباح الودائع الإسلامية</t>
+          <t>إيرادات الملكية الفكرية والتراخيص</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -5351,17 +5351,17 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>4700</t>
+          <t>4310</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Foreign exchange gain – realised</t>
+          <t>Intercompany IP and licence income</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>أرباح فروقات العملة المحققة</t>
+          <t>إيرادات ملكية فكرية من شركات المجموعة</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -5393,17 +5393,17 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>4710</t>
+          <t>4400</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Foreign exchange gain – unrealised</t>
+          <t>Dividend income</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>أرباح فروقات العملة غير المحققة</t>
+          <t>إيرادات توزيعات الأرباح</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -5435,17 +5435,17 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>4900</t>
+          <t>4500</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Non-compliant income (to purify)</t>
+          <t>Share of profit of associates</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>إيرادات غير متوافقة (للتطهير)</t>
+          <t>الحصة من أرباح الشركات الزميلة</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -5477,27 +5477,27 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>4600</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Expenses</t>
+          <t>Islamic deposit profit</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>المصروفات</t>
+          <t>أرباح الودائع الإسلامية</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -5519,22 +5519,22 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>5100</t>
+          <t>4700</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Salaries and benefits</t>
+          <t>Foreign exchange gain – realised</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>الرواتب والمزايا</t>
+          <t>أرباح فروقات العملة المحققة</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -5561,22 +5561,22 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>5110</t>
+          <t>4710</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>GOSI</t>
+          <t>Foreign exchange gain – unrealised</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>التأمينات الاجتماعية</t>
+          <t>أرباح فروقات العملة غير المحققة</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -5603,22 +5603,22 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>5200</t>
+          <t>4900</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Rent</t>
+          <t>Non-compliant income (to purify)</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>الإيجار</t>
+          <t>إيرادات غير متوافقة (للتطهير)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -5645,17 +5645,17 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>5300</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Professional fees</t>
+          <t>Expenses</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>الأتعاب المهنية</t>
+          <t>المصروفات</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -5665,7 +5665,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5687,17 +5687,17 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>5400</t>
+          <t>5100</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Depreciation</t>
+          <t>Salaries and benefits</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>الاستهلاك</t>
+          <t>الرواتب والمزايا</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -5729,17 +5729,17 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>5500</t>
+          <t>5110</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Repairs and maintenance</t>
+          <t>GOSI</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>الإصلاح والصيانة</t>
+          <t>التأمينات الاجتماعية</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -5771,17 +5771,17 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>5510</t>
+          <t>5120</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Vehicle fuel and running costs</t>
+          <t>End-of-service benefit expense</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>وقود ومصروفات السيارات</t>
+          <t>مصروف مكافأة نهاية الخدمة</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -5813,17 +5813,17 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>5600</t>
+          <t>5200</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Islamic financing cost</t>
+          <t>Rent</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>تكلفة التمويل الإسلامي</t>
+          <t>الإيجار</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -5855,17 +5855,17 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>5610</t>
+          <t>5300</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Conventional interest expense</t>
+          <t>Professional fees</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>مصروف فوائد تقليدية</t>
+          <t>الأتعاب المهنية</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -5885,7 +5885,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -5897,17 +5897,17 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>5700</t>
+          <t>5400</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Bank charges</t>
+          <t>Depreciation</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>رسوم بنكية</t>
+          <t>الاستهلاك</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -5939,17 +5939,17 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>5750</t>
+          <t>5500</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Foreign exchange loss – realised</t>
+          <t>Repairs and maintenance</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>خسائر فروقات العملة المحققة</t>
+          <t>الإصلاح والصيانة</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -5981,17 +5981,17 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>5760</t>
+          <t>5510</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Foreign exchange loss – unrealised</t>
+          <t>Vehicle fuel and running costs</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>خسائر فروقات العملة غير المحققة</t>
+          <t>وقود ومصروفات السيارات</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -6023,17 +6023,17 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>5770</t>
+          <t>5600</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Currency rounding differences</t>
+          <t>Islamic financing cost</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>فروقات تقريب العملات</t>
+          <t>تكلفة التمويل الإسلامي</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -6065,17 +6065,17 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>5800</t>
+          <t>5610</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Zakat</t>
+          <t>Conventional interest expense</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>الزكاة</t>
+          <t>مصروف فوائد تقليدية</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -6095,7 +6095,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -6107,17 +6107,17 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>5900</t>
+          <t>5700</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>General and administrative</t>
+          <t>Bank charges</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>مصروفات عمومية وإدارية</t>
+          <t>رسوم بنكية</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -6149,40 +6149,250 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
+          <t>5750</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Foreign exchange loss – realised</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>خسائر فروقات العملة المحققة</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Yes / نعم</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>5760</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Foreign exchange loss – unrealised</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>خسائر فروقات العملة غير المحققة</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Yes / نعم</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>5770</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Currency rounding differences</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>فروقات تقريب العملات</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Yes / نعم</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>5800</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Zakat</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>الزكاة</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Yes / نعم</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>5900</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>General and administrative</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>مصروفات عمومية وإدارية</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Yes / نعم</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
           <t>5920</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>Withholding tax borne (gross-up)</t>
         </is>
       </c>
-      <c r="C74" s="5" t="inlineStr">
+      <c r="C79" s="5" t="inlineStr">
         <is>
           <t>ضريبة استقطاع محملة على الشركة</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D79" t="inlineStr">
         <is>
           <t>expense</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
+      <c r="E79" t="inlineStr">
         <is>
           <t>Yes / نعم</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>No / لا</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>No / لا</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
         <is>
           <t>No / لا</t>
         </is>
@@ -6767,7 +6977,7 @@
       </c>
       <c r="U8" s="6" t="inlineStr">
         <is>
-          <t>1300</t>
+          <t>1230</t>
         </is>
       </c>
     </row>
@@ -6794,7 +7004,7 @@
       </c>
       <c r="U9" s="6" t="inlineStr">
         <is>
-          <t>1310</t>
+          <t>1240</t>
         </is>
       </c>
     </row>
@@ -6821,7 +7031,7 @@
       </c>
       <c r="U10" s="6" t="inlineStr">
         <is>
-          <t>1320</t>
+          <t>1300</t>
         </is>
       </c>
     </row>
@@ -6848,7 +7058,7 @@
       </c>
       <c r="U11" s="6" t="inlineStr">
         <is>
-          <t>1400</t>
+          <t>1310</t>
         </is>
       </c>
     </row>
@@ -6875,7 +7085,7 @@
       </c>
       <c r="U12" s="6" t="inlineStr">
         <is>
-          <t>1410</t>
+          <t>1320</t>
         </is>
       </c>
     </row>
@@ -6892,7 +7102,7 @@
       </c>
       <c r="U13" s="6" t="inlineStr">
         <is>
-          <t>1420</t>
+          <t>1400</t>
         </is>
       </c>
     </row>
@@ -6909,7 +7119,7 @@
       </c>
       <c r="U14" s="6" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>1410</t>
         </is>
       </c>
     </row>
@@ -6926,7 +7136,7 @@
       </c>
       <c r="U15" s="6" t="inlineStr">
         <is>
-          <t>1510</t>
+          <t>1420</t>
         </is>
       </c>
     </row>
@@ -6943,7 +7153,7 @@
       </c>
       <c r="U16" s="6" t="inlineStr">
         <is>
-          <t>1520</t>
+          <t>1500</t>
         </is>
       </c>
     </row>
@@ -6960,7 +7170,7 @@
       </c>
       <c r="U17" s="6" t="inlineStr">
         <is>
-          <t>1590</t>
+          <t>1510</t>
         </is>
       </c>
     </row>
@@ -6977,7 +7187,7 @@
       </c>
       <c r="U18" s="6" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>1520</t>
         </is>
       </c>
     </row>
@@ -6989,7 +7199,7 @@
       </c>
       <c r="U19" s="6" t="inlineStr">
         <is>
-          <t>2100</t>
+          <t>1590</t>
         </is>
       </c>
     </row>
@@ -7001,7 +7211,7 @@
       </c>
       <c r="U20" s="6" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>1600</t>
         </is>
       </c>
     </row>
@@ -7013,7 +7223,7 @@
       </c>
       <c r="U21" s="6" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>2100</t>
         </is>
       </c>
     </row>
@@ -7025,7 +7235,7 @@
       </c>
       <c r="U22" s="6" t="inlineStr">
         <is>
-          <t>2210</t>
+          <t>2110</t>
         </is>
       </c>
     </row>
@@ -7037,7 +7247,7 @@
       </c>
       <c r="U23" s="6" t="inlineStr">
         <is>
-          <t>2220</t>
+          <t>2200</t>
         </is>
       </c>
     </row>
@@ -7049,7 +7259,7 @@
       </c>
       <c r="U24" s="6" t="inlineStr">
         <is>
-          <t>2300</t>
+          <t>2210</t>
         </is>
       </c>
     </row>
@@ -7061,7 +7271,7 @@
       </c>
       <c r="U25" s="6" t="inlineStr">
         <is>
-          <t>2400</t>
+          <t>2220</t>
         </is>
       </c>
     </row>
@@ -7073,7 +7283,7 @@
       </c>
       <c r="U26" s="6" t="inlineStr">
         <is>
-          <t>2410</t>
+          <t>2300</t>
         </is>
       </c>
     </row>
@@ -7085,7 +7295,7 @@
       </c>
       <c r="U27" s="6" t="inlineStr">
         <is>
-          <t>2500</t>
+          <t>2330</t>
         </is>
       </c>
     </row>
@@ -7097,7 +7307,7 @@
       </c>
       <c r="U28" s="6" t="inlineStr">
         <is>
-          <t>2600</t>
+          <t>2340</t>
         </is>
       </c>
     </row>
@@ -7109,7 +7319,7 @@
       </c>
       <c r="U29" s="6" t="inlineStr">
         <is>
-          <t>3100</t>
+          <t>2400</t>
         </is>
       </c>
     </row>
@@ -7121,7 +7331,7 @@
       </c>
       <c r="U30" s="6" t="inlineStr">
         <is>
-          <t>3200</t>
+          <t>2410</t>
         </is>
       </c>
     </row>
@@ -7133,7 +7343,7 @@
       </c>
       <c r="U31" s="6" t="inlineStr">
         <is>
-          <t>3300</t>
+          <t>2500</t>
         </is>
       </c>
     </row>
@@ -7145,7 +7355,7 @@
       </c>
       <c r="U32" s="6" t="inlineStr">
         <is>
-          <t>3900</t>
+          <t>2600</t>
         </is>
       </c>
     </row>
@@ -7157,7 +7367,7 @@
       </c>
       <c r="U33" s="6" t="inlineStr">
         <is>
-          <t>4100</t>
+          <t>3100</t>
         </is>
       </c>
     </row>
@@ -7169,7 +7379,7 @@
       </c>
       <c r="U34" s="6" t="inlineStr">
         <is>
-          <t>4110</t>
+          <t>3200</t>
         </is>
       </c>
     </row>
@@ -7181,7 +7391,7 @@
       </c>
       <c r="U35" s="6" t="inlineStr">
         <is>
-          <t>4120</t>
+          <t>3300</t>
         </is>
       </c>
     </row>
@@ -7193,7 +7403,7 @@
       </c>
       <c r="U36" s="6" t="inlineStr">
         <is>
-          <t>4200</t>
+          <t>3900</t>
         </is>
       </c>
     </row>
@@ -7205,7 +7415,7 @@
       </c>
       <c r="U37" s="6" t="inlineStr">
         <is>
-          <t>4210</t>
+          <t>4100</t>
         </is>
       </c>
     </row>
@@ -7217,7 +7427,7 @@
       </c>
       <c r="U38" s="6" t="inlineStr">
         <is>
-          <t>4220</t>
+          <t>4110</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7439,7 @@
       </c>
       <c r="U39" s="6" t="inlineStr">
         <is>
-          <t>4230</t>
+          <t>4120</t>
         </is>
       </c>
     </row>
@@ -7241,7 +7451,7 @@
       </c>
       <c r="U40" s="6" t="inlineStr">
         <is>
-          <t>4240</t>
+          <t>4200</t>
         </is>
       </c>
     </row>
@@ -7253,7 +7463,7 @@
       </c>
       <c r="U41" s="6" t="inlineStr">
         <is>
-          <t>4300</t>
+          <t>4210</t>
         </is>
       </c>
     </row>
@@ -7265,7 +7475,7 @@
       </c>
       <c r="U42" s="6" t="inlineStr">
         <is>
-          <t>4310</t>
+          <t>4220</t>
         </is>
       </c>
     </row>
@@ -7277,7 +7487,7 @@
       </c>
       <c r="U43" s="6" t="inlineStr">
         <is>
-          <t>4400</t>
+          <t>4230</t>
         </is>
       </c>
     </row>
@@ -7289,7 +7499,7 @@
       </c>
       <c r="U44" s="6" t="inlineStr">
         <is>
-          <t>4500</t>
+          <t>4240</t>
         </is>
       </c>
     </row>
@@ -7301,7 +7511,7 @@
       </c>
       <c r="U45" s="6" t="inlineStr">
         <is>
-          <t>4600</t>
+          <t>4300</t>
         </is>
       </c>
     </row>
@@ -7313,7 +7523,7 @@
       </c>
       <c r="U46" s="6" t="inlineStr">
         <is>
-          <t>4700</t>
+          <t>4310</t>
         </is>
       </c>
     </row>
@@ -7325,7 +7535,7 @@
       </c>
       <c r="U47" s="6" t="inlineStr">
         <is>
-          <t>4710</t>
+          <t>4400</t>
         </is>
       </c>
     </row>
@@ -7337,7 +7547,7 @@
       </c>
       <c r="U48" s="6" t="inlineStr">
         <is>
-          <t>4900</t>
+          <t>4500</t>
         </is>
       </c>
     </row>
@@ -7349,7 +7559,7 @@
       </c>
       <c r="U49" s="6" t="inlineStr">
         <is>
-          <t>5100</t>
+          <t>4600</t>
         </is>
       </c>
     </row>
@@ -7361,7 +7571,7 @@
       </c>
       <c r="U50" s="6" t="inlineStr">
         <is>
-          <t>5110</t>
+          <t>4700</t>
         </is>
       </c>
     </row>
@@ -7373,7 +7583,7 @@
       </c>
       <c r="U51" s="6" t="inlineStr">
         <is>
-          <t>5200</t>
+          <t>4710</t>
         </is>
       </c>
     </row>
@@ -7385,7 +7595,7 @@
       </c>
       <c r="U52" s="6" t="inlineStr">
         <is>
-          <t>5300</t>
+          <t>4900</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7607,7 @@
       </c>
       <c r="U53" s="6" t="inlineStr">
         <is>
-          <t>5400</t>
+          <t>5100</t>
         </is>
       </c>
     </row>
@@ -7409,7 +7619,7 @@
       </c>
       <c r="U54" s="6" t="inlineStr">
         <is>
-          <t>5500</t>
+          <t>5110</t>
         </is>
       </c>
     </row>
@@ -7421,7 +7631,7 @@
       </c>
       <c r="U55" s="6" t="inlineStr">
         <is>
-          <t>5510</t>
+          <t>5120</t>
         </is>
       </c>
     </row>
@@ -7433,7 +7643,7 @@
       </c>
       <c r="U56" s="6" t="inlineStr">
         <is>
-          <t>5600</t>
+          <t>5200</t>
         </is>
       </c>
     </row>
@@ -7445,7 +7655,7 @@
       </c>
       <c r="U57" s="6" t="inlineStr">
         <is>
-          <t>5610</t>
+          <t>5300</t>
         </is>
       </c>
     </row>
@@ -7457,7 +7667,7 @@
       </c>
       <c r="U58" s="6" t="inlineStr">
         <is>
-          <t>5700</t>
+          <t>5400</t>
         </is>
       </c>
     </row>
@@ -7469,7 +7679,7 @@
       </c>
       <c r="U59" s="6" t="inlineStr">
         <is>
-          <t>5750</t>
+          <t>5500</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7691,7 @@
       </c>
       <c r="U60" s="6" t="inlineStr">
         <is>
-          <t>5760</t>
+          <t>5510</t>
         </is>
       </c>
     </row>
@@ -7493,7 +7703,7 @@
       </c>
       <c r="U61" s="6" t="inlineStr">
         <is>
-          <t>5770</t>
+          <t>5600</t>
         </is>
       </c>
     </row>
@@ -7505,7 +7715,7 @@
       </c>
       <c r="U62" s="6" t="inlineStr">
         <is>
-          <t>5800</t>
+          <t>5610</t>
         </is>
       </c>
     </row>
@@ -7517,7 +7727,7 @@
       </c>
       <c r="U63" s="6" t="inlineStr">
         <is>
-          <t>5900</t>
+          <t>5700</t>
         </is>
       </c>
     </row>
@@ -7529,7 +7739,7 @@
       </c>
       <c r="U64" s="6" t="inlineStr">
         <is>
-          <t>5920</t>
+          <t>5750</t>
         </is>
       </c>
     </row>
@@ -7539,6 +7749,11 @@
           <t>EE</t>
         </is>
       </c>
+      <c r="U65" s="6" t="inlineStr">
+        <is>
+          <t>5760</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="T66" s="6" t="inlineStr">
@@ -7546,6 +7761,11 @@
           <t>EG</t>
         </is>
       </c>
+      <c r="U66" s="6" t="inlineStr">
+        <is>
+          <t>5770</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="T67" s="6" t="inlineStr">
@@ -7553,6 +7773,11 @@
           <t>EH</t>
         </is>
       </c>
+      <c r="U67" s="6" t="inlineStr">
+        <is>
+          <t>5800</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="T68" s="6" t="inlineStr">
@@ -7560,11 +7785,21 @@
           <t>ER</t>
         </is>
       </c>
+      <c r="U68" s="6" t="inlineStr">
+        <is>
+          <t>5900</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="T69" s="6" t="inlineStr">
         <is>
           <t>ES</t>
+        </is>
+      </c>
+      <c r="U69" s="6" t="inlineStr">
+        <is>
+          <t>5920</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate the migration workbook and allow-list the port's sale lookup
The workbook's ERP chart sheet lists every template account, so it now shows the
bai' ajel accounts 1241, 1250 and 4610 (and 5930, added to the template meanwhile).
deferred_sale_of is read only by the payroll invoicing port for a contract payroll
already holds; it returns amounts and status, no personal data, so it is reviewed
onto the access-scan allow-list instead of taking a right of its own.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVy7Y2kCiQ1NrNgFBo2Zhn
</commit_message>
<xml_diff>
--- a/docs/migration/almiras-migration-workbook.xlsx
+++ b/docs/migration/almiras-migration-workbook.xlsx
@@ -44,7 +44,7 @@
     <definedName name="L_checklist_status">'Lists'!$R$2:$R$4</definedName>
     <definedName name="L_currency">'Lists'!$S$2:$S$18</definedName>
     <definedName name="L_country">'Lists'!$T$2:$T$250</definedName>
-    <definedName name="L_erp_code">'Lists'!$U$2:$U$69</definedName>
+    <definedName name="L_erp_code">'Lists'!$U$2:$U$73</definedName>
     <definedName name="L_entity">'Entities'!$A$6:$A$2005</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3179,7 +3179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3671,17 +3671,17 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>1300</t>
+          <t>1241</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Sharia-compliant deposits (e.g. murabaha, wakala)</t>
+          <t>Deferred bai' ajel profit (contra 1240)</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>ودائع متوافقة مع الشريعة</t>
+          <t>أرباح البيع الآجل المؤجلة</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -3713,17 +3713,17 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>1310</t>
+          <t>1250</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>VAT input</t>
+          <t>Assets acquired for employee deferred sale</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>ضريبة القيمة المضافة - مدخلات</t>
+          <t>أصول مشتراة للبيع الآجل للموظفين</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -3755,17 +3755,17 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>1320</t>
+          <t>1300</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Prepayments</t>
+          <t>Sharia-compliant deposits (e.g. murabaha, wakala)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>مصروفات مدفوعة مقدماً</t>
+          <t>ودائع متوافقة مع الشريعة</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -3797,17 +3797,17 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>1400</t>
+          <t>1310</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Investments in subsidiaries</t>
+          <t>VAT input</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>استثمارات في شركات تابعة</t>
+          <t>ضريبة القيمة المضافة - مدخلات</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -3839,17 +3839,17 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>1410</t>
+          <t>1320</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Investments in associates (equity method)</t>
+          <t>Prepayments</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>استثمارات في شركات زميلة</t>
+          <t>مصروفات مدفوعة مقدماً</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -3881,17 +3881,17 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>1420</t>
+          <t>1400</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Other equity investments</t>
+          <t>Investments in subsidiaries</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>استثمارات حقوق ملكية أخرى</t>
+          <t>استثمارات في شركات تابعة</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -3923,17 +3923,17 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>1410</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Property, plant and equipment</t>
+          <t>Investments in associates (equity method)</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>الممتلكات والآلات والمعدات</t>
+          <t>استثمارات في شركات زميلة</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -3965,17 +3965,17 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>1510</t>
+          <t>1420</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Investment property (rental assets)</t>
+          <t>Other equity investments</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>عقارات استثمارية</t>
+          <t>استثمارات حقوق ملكية أخرى</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -4007,17 +4007,17 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>1520</t>
+          <t>1500</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Vehicles</t>
+          <t>Property, plant and equipment</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>السيارات</t>
+          <t>الممتلكات والآلات والمعدات</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -4049,17 +4049,17 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>1590</t>
+          <t>1510</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Accumulated depreciation</t>
+          <t>Investment property (rental assets)</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>مجمع الاستهلاك</t>
+          <t>عقارات استثمارية</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -4091,17 +4091,17 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>1520</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Intangible assets and IP</t>
+          <t>Vehicles</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>الأصول غير الملموسة والملكية الفكرية</t>
+          <t>السيارات</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -4133,27 +4133,27 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>1590</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Liabilities</t>
+          <t>Accumulated depreciation</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>الالتزامات</t>
+          <t>مجمع الاستهلاك</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>liability</t>
+          <t>asset</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -4175,22 +4175,22 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>2100</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Trade payables</t>
+          <t>Intangible assets and IP</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>الذمم الدائنة التجارية</t>
+          <t>الأصول غير الملموسة والملكية الفكرية</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>liability</t>
+          <t>asset</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -4210,24 +4210,24 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Due to group entities</t>
+          <t>Liabilities</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>مستحق لشركات المجموعة</t>
+          <t>الالتزامات</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -4237,12 +4237,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -4252,24 +4252,24 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>2100</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>VAT output</t>
+          <t>Trade payables</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>ضريبة القيمة المضافة - مخرجات</t>
+          <t>الذمم الدائنة التجارية</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -4294,24 +4294,24 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>2210</t>
+          <t>2110</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Zakat payable</t>
+          <t>Due to group entities</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>الزكاة المستحقة</t>
+          <t>مستحق لشركات المجموعة</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -4326,7 +4326,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -4336,24 +4336,24 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>2220</t>
+          <t>2200</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Withholding tax payable</t>
+          <t>VAT output</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>ضريبة الاستقطاع المستحقة</t>
+          <t>ضريبة القيمة المضافة - مخرجات</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -4385,17 +4385,17 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>2300</t>
+          <t>2210</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Accrued expenses</t>
+          <t>Zakat payable</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>مصروفات مستحقة</t>
+          <t>الزكاة المستحقة</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -4427,17 +4427,17 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>2330</t>
+          <t>2220</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Salaries payable</t>
+          <t>Withholding tax payable</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>رواتب مستحقة</t>
+          <t>ضريبة الاستقطاع المستحقة</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -4469,17 +4469,17 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>2340</t>
+          <t>2300</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>GOSI payable</t>
+          <t>Accrued expenses</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>اشتراكات التأمينات الاجتماعية المستحقة</t>
+          <t>مصروفات مستحقة</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4511,17 +4511,17 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>2400</t>
+          <t>2330</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Islamic financing (murabaha, tawarruq)</t>
+          <t>Salaries payable</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>تمويل إسلامي</t>
+          <t>رواتب مستحقة</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -4553,17 +4553,17 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>2410</t>
+          <t>2340</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Conventional interest-bearing loans</t>
+          <t>GOSI payable</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>قروض تقليدية بفائدة</t>
+          <t>اشتراكات التأمينات الاجتماعية المستحقة</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -4595,17 +4595,17 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>2500</t>
+          <t>2400</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>End-of-service provision</t>
+          <t>Islamic financing (murabaha, tawarruq)</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>مخصص مكافأة نهاية الخدمة</t>
+          <t>تمويل إسلامي</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -4637,17 +4637,17 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>2600</t>
+          <t>2410</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Charity payable (purification)</t>
+          <t>Conventional interest-bearing loans</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>مبالغ مستحقة للتطهير</t>
+          <t>قروض تقليدية بفائدة</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -4667,7 +4667,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -4679,27 +4679,27 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>3000</t>
+          <t>2500</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Equity</t>
+          <t>End-of-service provision</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>حقوق الملكية</t>
+          <t>مخصص مكافأة نهاية الخدمة</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>equity</t>
+          <t>liability</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4721,22 +4721,22 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>3100</t>
+          <t>2600</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Share capital</t>
+          <t>Charity payable (purification)</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>رأس المال</t>
+          <t>مبالغ مستحقة للتطهير</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>equity</t>
+          <t>liability</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -4763,17 +4763,17 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>3200</t>
+          <t>3000</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Statutory reserve</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>الاحتياطي النظامي</t>
+          <t>حقوق الملكية</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -4783,7 +4783,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4805,17 +4805,17 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>3300</t>
+          <t>3100</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Retained earnings</t>
+          <t>Share capital</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>الأرباح المبقاة</t>
+          <t>رأس المال</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -4847,17 +4847,17 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>3400</t>
+          <t>3200</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Foreign currency translation reserve</t>
+          <t>Statutory reserve</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>احتياطي ترجمة العملات الأجنبية</t>
+          <t>الاحتياطي النظامي</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4867,7 +4867,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -4889,17 +4889,17 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>3900</t>
+          <t>3300</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Opening balance equity (migration)</t>
+          <t>Retained earnings</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>حقوق ملكية الأرصدة الافتتاحية</t>
+          <t>الأرباح المبقاة</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -4931,22 +4931,22 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>4000</t>
+          <t>3400</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Foreign currency translation reserve</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>الإيرادات</t>
+          <t>احتياطي ترجمة العملات الأجنبية</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>income</t>
+          <t>equity</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -4973,22 +4973,22 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>4100</t>
+          <t>3900</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Rental income</t>
+          <t>Opening balance equity (migration)</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>إيرادات الإيجار</t>
+          <t>حقوق ملكية الأرصدة الافتتاحية</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>income</t>
+          <t>equity</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -5015,17 +5015,17 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>4110</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Intercompany rental income</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>إيرادات إيجار من شركات المجموعة</t>
+          <t>الإيرادات</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -5035,7 +5035,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -5057,17 +5057,17 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>4120</t>
+          <t>4100</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Residential rental income (VAT-exempt)</t>
+          <t>Rental income</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>إيرادات الإيجار السكني (معفاة)</t>
+          <t>إيرادات الإيجار</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5099,17 +5099,17 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>4200</t>
+          <t>4110</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Secondment and consulting income</t>
+          <t>Intercompany rental income</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>إيرادات الإعارة والاستشارات</t>
+          <t>إيرادات إيجار من شركات المجموعة</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5141,17 +5141,17 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>4210</t>
+          <t>4120</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Intercompany service income</t>
+          <t>Residential rental income (VAT-exempt)</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>إيرادات خدمات من شركات المجموعة</t>
+          <t>إيرادات الإيجار السكني (معفاة)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5183,17 +5183,17 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>4220</t>
+          <t>4200</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Management fee income</t>
+          <t>Secondment and consulting income</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>إيرادات رسوم الإدارة</t>
+          <t>إيرادات الإعارة والاستشارات</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -5225,17 +5225,17 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>4230</t>
+          <t>4210</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Service charge income</t>
+          <t>Intercompany service income</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>إيرادات رسوم الخدمات المشتركة</t>
+          <t>إيرادات خدمات من شركات المجموعة</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -5267,17 +5267,17 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>4240</t>
+          <t>4220</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Service fee income</t>
+          <t>Management fee income</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>إيرادات أتعاب الخدمات</t>
+          <t>إيرادات رسوم الإدارة</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -5309,17 +5309,17 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>4300</t>
+          <t>4230</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>IP and licence income</t>
+          <t>Service charge income</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>إيرادات الملكية الفكرية والتراخيص</t>
+          <t>إيرادات رسوم الخدمات المشتركة</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -5351,17 +5351,17 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>4310</t>
+          <t>4240</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Intercompany IP and licence income</t>
+          <t>Service fee income</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>إيرادات ملكية فكرية من شركات المجموعة</t>
+          <t>إيرادات أتعاب الخدمات</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -5393,17 +5393,17 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>4400</t>
+          <t>4300</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Dividend income</t>
+          <t>IP and licence income</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>إيرادات توزيعات الأرباح</t>
+          <t>إيرادات الملكية الفكرية والتراخيص</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -5435,17 +5435,17 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>4500</t>
+          <t>4310</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Share of profit of associates</t>
+          <t>Intercompany IP and licence income</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>الحصة من أرباح الشركات الزميلة</t>
+          <t>إيرادات ملكية فكرية من شركات المجموعة</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -5477,17 +5477,17 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>4600</t>
+          <t>4400</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Islamic deposit profit</t>
+          <t>Dividend income</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>أرباح الودائع الإسلامية</t>
+          <t>إيرادات توزيعات الأرباح</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -5519,17 +5519,17 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>4700</t>
+          <t>4500</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Foreign exchange gain – realised</t>
+          <t>Share of profit of associates</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>أرباح فروقات العملة المحققة</t>
+          <t>الحصة من أرباح الشركات الزميلة</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -5561,17 +5561,17 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>4710</t>
+          <t>4600</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Foreign exchange gain – unrealised</t>
+          <t>Islamic deposit profit</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>أرباح فروقات العملة غير المحققة</t>
+          <t>أرباح الودائع الإسلامية</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -5603,17 +5603,17 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>4900</t>
+          <t>4610</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Non-compliant income (to purify)</t>
+          <t>Bai' ajel profit income</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>إيرادات غير متوافقة (للتطهير)</t>
+          <t>إيرادات أرباح البيع الآجل</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -5645,27 +5645,27 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>4700</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Expenses</t>
+          <t>Foreign exchange gain – realised</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>المصروفات</t>
+          <t>أرباح فروقات العملة المحققة</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5687,22 +5687,22 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>5100</t>
+          <t>4710</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Salaries and benefits</t>
+          <t>Foreign exchange gain – unrealised</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>الرواتب والمزايا</t>
+          <t>أرباح فروقات العملة غير المحققة</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -5729,22 +5729,22 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>5110</t>
+          <t>4900</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>GOSI</t>
+          <t>Non-compliant income (to purify)</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>التأمينات الاجتماعية</t>
+          <t>إيرادات غير متوافقة (للتطهير)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>expense</t>
+          <t>income</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -5771,17 +5771,17 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>5120</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>End-of-service benefit expense</t>
+          <t>Expenses</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>مصروف مكافأة نهاية الخدمة</t>
+          <t>المصروفات</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -5791,7 +5791,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -5813,17 +5813,17 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>5200</t>
+          <t>5100</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Rent</t>
+          <t>Salaries and benefits</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>الإيجار</t>
+          <t>الرواتب والمزايا</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -5855,17 +5855,17 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>5300</t>
+          <t>5110</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Professional fees</t>
+          <t>GOSI</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>الأتعاب المهنية</t>
+          <t>التأمينات الاجتماعية</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -5897,17 +5897,17 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>5400</t>
+          <t>5120</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Depreciation</t>
+          <t>End-of-service benefit expense</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>الاستهلاك</t>
+          <t>مصروف مكافأة نهاية الخدمة</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -5939,17 +5939,17 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>5500</t>
+          <t>5200</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Repairs and maintenance</t>
+          <t>Rent</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>الإصلاح والصيانة</t>
+          <t>الإيجار</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -5981,17 +5981,17 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>5510</t>
+          <t>5300</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Vehicle fuel and running costs</t>
+          <t>Professional fees</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>وقود ومصروفات السيارات</t>
+          <t>الأتعاب المهنية</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -6023,17 +6023,17 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>5600</t>
+          <t>5400</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Islamic financing cost</t>
+          <t>Depreciation</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>تكلفة التمويل الإسلامي</t>
+          <t>الاستهلاك</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -6065,17 +6065,17 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>5610</t>
+          <t>5500</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Conventional interest expense</t>
+          <t>Repairs and maintenance</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>مصروف فوائد تقليدية</t>
+          <t>الإصلاح والصيانة</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -6095,7 +6095,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Yes / نعم</t>
+          <t>No / لا</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -6107,17 +6107,17 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>5700</t>
+          <t>5510</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Bank charges</t>
+          <t>Vehicle fuel and running costs</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>رسوم بنكية</t>
+          <t>وقود ومصروفات السيارات</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -6149,17 +6149,17 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>5750</t>
+          <t>5600</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Foreign exchange loss – realised</t>
+          <t>Islamic financing cost</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>خسائر فروقات العملة المحققة</t>
+          <t>تكلفة التمويل الإسلامي</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -6191,17 +6191,17 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>5760</t>
+          <t>5610</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Foreign exchange loss – unrealised</t>
+          <t>Conventional interest expense</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>خسائر فروقات العملة غير المحققة</t>
+          <t>مصروف فوائد تقليدية</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -6221,7 +6221,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>No / لا</t>
+          <t>Yes / نعم</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -6233,17 +6233,17 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>5770</t>
+          <t>5700</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Currency rounding differences</t>
+          <t>Bank charges</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>فروقات تقريب العملات</t>
+          <t>رسوم بنكية</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -6275,17 +6275,17 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>5800</t>
+          <t>5750</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Zakat</t>
+          <t>Foreign exchange loss – realised</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>الزكاة</t>
+          <t>خسائر فروقات العملة المحققة</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -6317,17 +6317,17 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>5900</t>
+          <t>5760</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>General and administrative</t>
+          <t>Foreign exchange loss – unrealised</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>مصروفات عمومية وإدارية</t>
+          <t>خسائر فروقات العملة غير المحققة</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -6359,40 +6359,208 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
+          <t>5770</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Currency rounding differences</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>فروقات تقريب العملات</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Yes / نعم</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>5800</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Zakat</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>الزكاة</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Yes / نعم</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>5900</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>General and administrative</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>مصروفات عمومية وإدارية</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Yes / نعم</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
           <t>5920</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B82" t="inlineStr">
         <is>
           <t>Withholding tax borne (gross-up)</t>
         </is>
       </c>
-      <c r="C79" s="5" t="inlineStr">
+      <c r="C82" s="5" t="inlineStr">
         <is>
           <t>ضريبة استقطاع محملة على الشركة</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="D82" t="inlineStr">
         <is>
           <t>expense</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
+      <c r="E82" t="inlineStr">
         <is>
           <t>Yes / نعم</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>No / لا</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>No / لا</t>
-        </is>
-      </c>
-      <c r="H79" t="inlineStr">
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>5930</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>GOSI late-payment fines</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>غرامات تأخير التأمينات</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>expense</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Yes / نعم</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>No / لا</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
         <is>
           <t>No / لا</t>
         </is>
@@ -7031,7 +7199,7 @@
       </c>
       <c r="U10" s="6" t="inlineStr">
         <is>
-          <t>1300</t>
+          <t>1241</t>
         </is>
       </c>
     </row>
@@ -7058,7 +7226,7 @@
       </c>
       <c r="U11" s="6" t="inlineStr">
         <is>
-          <t>1310</t>
+          <t>1250</t>
         </is>
       </c>
     </row>
@@ -7085,7 +7253,7 @@
       </c>
       <c r="U12" s="6" t="inlineStr">
         <is>
-          <t>1320</t>
+          <t>1300</t>
         </is>
       </c>
     </row>
@@ -7102,7 +7270,7 @@
       </c>
       <c r="U13" s="6" t="inlineStr">
         <is>
-          <t>1400</t>
+          <t>1310</t>
         </is>
       </c>
     </row>
@@ -7119,7 +7287,7 @@
       </c>
       <c r="U14" s="6" t="inlineStr">
         <is>
-          <t>1410</t>
+          <t>1320</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7304,7 @@
       </c>
       <c r="U15" s="6" t="inlineStr">
         <is>
-          <t>1420</t>
+          <t>1400</t>
         </is>
       </c>
     </row>
@@ -7153,7 +7321,7 @@
       </c>
       <c r="U16" s="6" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>1410</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7338,7 @@
       </c>
       <c r="U17" s="6" t="inlineStr">
         <is>
-          <t>1510</t>
+          <t>1420</t>
         </is>
       </c>
     </row>
@@ -7187,7 +7355,7 @@
       </c>
       <c r="U18" s="6" t="inlineStr">
         <is>
-          <t>1520</t>
+          <t>1500</t>
         </is>
       </c>
     </row>
@@ -7199,7 +7367,7 @@
       </c>
       <c r="U19" s="6" t="inlineStr">
         <is>
-          <t>1590</t>
+          <t>1510</t>
         </is>
       </c>
     </row>
@@ -7211,7 +7379,7 @@
       </c>
       <c r="U20" s="6" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>1520</t>
         </is>
       </c>
     </row>
@@ -7223,7 +7391,7 @@
       </c>
       <c r="U21" s="6" t="inlineStr">
         <is>
-          <t>2100</t>
+          <t>1590</t>
         </is>
       </c>
     </row>
@@ -7235,7 +7403,7 @@
       </c>
       <c r="U22" s="6" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>1600</t>
         </is>
       </c>
     </row>
@@ -7247,7 +7415,7 @@
       </c>
       <c r="U23" s="6" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>2100</t>
         </is>
       </c>
     </row>
@@ -7259,7 +7427,7 @@
       </c>
       <c r="U24" s="6" t="inlineStr">
         <is>
-          <t>2210</t>
+          <t>2110</t>
         </is>
       </c>
     </row>
@@ -7271,7 +7439,7 @@
       </c>
       <c r="U25" s="6" t="inlineStr">
         <is>
-          <t>2220</t>
+          <t>2200</t>
         </is>
       </c>
     </row>
@@ -7283,7 +7451,7 @@
       </c>
       <c r="U26" s="6" t="inlineStr">
         <is>
-          <t>2300</t>
+          <t>2210</t>
         </is>
       </c>
     </row>
@@ -7295,7 +7463,7 @@
       </c>
       <c r="U27" s="6" t="inlineStr">
         <is>
-          <t>2330</t>
+          <t>2220</t>
         </is>
       </c>
     </row>
@@ -7307,7 +7475,7 @@
       </c>
       <c r="U28" s="6" t="inlineStr">
         <is>
-          <t>2340</t>
+          <t>2300</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7487,7 @@
       </c>
       <c r="U29" s="6" t="inlineStr">
         <is>
-          <t>2400</t>
+          <t>2330</t>
         </is>
       </c>
     </row>
@@ -7331,7 +7499,7 @@
       </c>
       <c r="U30" s="6" t="inlineStr">
         <is>
-          <t>2410</t>
+          <t>2340</t>
         </is>
       </c>
     </row>
@@ -7343,7 +7511,7 @@
       </c>
       <c r="U31" s="6" t="inlineStr">
         <is>
-          <t>2500</t>
+          <t>2400</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7523,7 @@
       </c>
       <c r="U32" s="6" t="inlineStr">
         <is>
-          <t>2600</t>
+          <t>2410</t>
         </is>
       </c>
     </row>
@@ -7367,7 +7535,7 @@
       </c>
       <c r="U33" s="6" t="inlineStr">
         <is>
-          <t>3100</t>
+          <t>2500</t>
         </is>
       </c>
     </row>
@@ -7379,7 +7547,7 @@
       </c>
       <c r="U34" s="6" t="inlineStr">
         <is>
-          <t>3200</t>
+          <t>2600</t>
         </is>
       </c>
     </row>
@@ -7391,7 +7559,7 @@
       </c>
       <c r="U35" s="6" t="inlineStr">
         <is>
-          <t>3300</t>
+          <t>3100</t>
         </is>
       </c>
     </row>
@@ -7403,7 +7571,7 @@
       </c>
       <c r="U36" s="6" t="inlineStr">
         <is>
-          <t>3900</t>
+          <t>3200</t>
         </is>
       </c>
     </row>
@@ -7415,7 +7583,7 @@
       </c>
       <c r="U37" s="6" t="inlineStr">
         <is>
-          <t>4100</t>
+          <t>3300</t>
         </is>
       </c>
     </row>
@@ -7427,7 +7595,7 @@
       </c>
       <c r="U38" s="6" t="inlineStr">
         <is>
-          <t>4110</t>
+          <t>3900</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7607,7 @@
       </c>
       <c r="U39" s="6" t="inlineStr">
         <is>
-          <t>4120</t>
+          <t>4100</t>
         </is>
       </c>
     </row>
@@ -7451,7 +7619,7 @@
       </c>
       <c r="U40" s="6" t="inlineStr">
         <is>
-          <t>4200</t>
+          <t>4110</t>
         </is>
       </c>
     </row>
@@ -7463,7 +7631,7 @@
       </c>
       <c r="U41" s="6" t="inlineStr">
         <is>
-          <t>4210</t>
+          <t>4120</t>
         </is>
       </c>
     </row>
@@ -7475,7 +7643,7 @@
       </c>
       <c r="U42" s="6" t="inlineStr">
         <is>
-          <t>4220</t>
+          <t>4200</t>
         </is>
       </c>
     </row>
@@ -7487,7 +7655,7 @@
       </c>
       <c r="U43" s="6" t="inlineStr">
         <is>
-          <t>4230</t>
+          <t>4210</t>
         </is>
       </c>
     </row>
@@ -7499,7 +7667,7 @@
       </c>
       <c r="U44" s="6" t="inlineStr">
         <is>
-          <t>4240</t>
+          <t>4220</t>
         </is>
       </c>
     </row>
@@ -7511,7 +7679,7 @@
       </c>
       <c r="U45" s="6" t="inlineStr">
         <is>
-          <t>4300</t>
+          <t>4230</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7691,7 @@
       </c>
       <c r="U46" s="6" t="inlineStr">
         <is>
-          <t>4310</t>
+          <t>4240</t>
         </is>
       </c>
     </row>
@@ -7535,7 +7703,7 @@
       </c>
       <c r="U47" s="6" t="inlineStr">
         <is>
-          <t>4400</t>
+          <t>4300</t>
         </is>
       </c>
     </row>
@@ -7547,7 +7715,7 @@
       </c>
       <c r="U48" s="6" t="inlineStr">
         <is>
-          <t>4500</t>
+          <t>4310</t>
         </is>
       </c>
     </row>
@@ -7559,7 +7727,7 @@
       </c>
       <c r="U49" s="6" t="inlineStr">
         <is>
-          <t>4600</t>
+          <t>4400</t>
         </is>
       </c>
     </row>
@@ -7571,7 +7739,7 @@
       </c>
       <c r="U50" s="6" t="inlineStr">
         <is>
-          <t>4700</t>
+          <t>4500</t>
         </is>
       </c>
     </row>
@@ -7583,7 +7751,7 @@
       </c>
       <c r="U51" s="6" t="inlineStr">
         <is>
-          <t>4710</t>
+          <t>4600</t>
         </is>
       </c>
     </row>
@@ -7595,7 +7763,7 @@
       </c>
       <c r="U52" s="6" t="inlineStr">
         <is>
-          <t>4900</t>
+          <t>4610</t>
         </is>
       </c>
     </row>
@@ -7607,7 +7775,7 @@
       </c>
       <c r="U53" s="6" t="inlineStr">
         <is>
-          <t>5100</t>
+          <t>4700</t>
         </is>
       </c>
     </row>
@@ -7619,7 +7787,7 @@
       </c>
       <c r="U54" s="6" t="inlineStr">
         <is>
-          <t>5110</t>
+          <t>4710</t>
         </is>
       </c>
     </row>
@@ -7631,7 +7799,7 @@
       </c>
       <c r="U55" s="6" t="inlineStr">
         <is>
-          <t>5120</t>
+          <t>4900</t>
         </is>
       </c>
     </row>
@@ -7643,7 +7811,7 @@
       </c>
       <c r="U56" s="6" t="inlineStr">
         <is>
-          <t>5200</t>
+          <t>5100</t>
         </is>
       </c>
     </row>
@@ -7655,7 +7823,7 @@
       </c>
       <c r="U57" s="6" t="inlineStr">
         <is>
-          <t>5300</t>
+          <t>5110</t>
         </is>
       </c>
     </row>
@@ -7667,7 +7835,7 @@
       </c>
       <c r="U58" s="6" t="inlineStr">
         <is>
-          <t>5400</t>
+          <t>5120</t>
         </is>
       </c>
     </row>
@@ -7679,7 +7847,7 @@
       </c>
       <c r="U59" s="6" t="inlineStr">
         <is>
-          <t>5500</t>
+          <t>5200</t>
         </is>
       </c>
     </row>
@@ -7691,7 +7859,7 @@
       </c>
       <c r="U60" s="6" t="inlineStr">
         <is>
-          <t>5510</t>
+          <t>5300</t>
         </is>
       </c>
     </row>
@@ -7703,7 +7871,7 @@
       </c>
       <c r="U61" s="6" t="inlineStr">
         <is>
-          <t>5600</t>
+          <t>5400</t>
         </is>
       </c>
     </row>
@@ -7715,7 +7883,7 @@
       </c>
       <c r="U62" s="6" t="inlineStr">
         <is>
-          <t>5610</t>
+          <t>5500</t>
         </is>
       </c>
     </row>
@@ -7727,7 +7895,7 @@
       </c>
       <c r="U63" s="6" t="inlineStr">
         <is>
-          <t>5700</t>
+          <t>5510</t>
         </is>
       </c>
     </row>
@@ -7739,7 +7907,7 @@
       </c>
       <c r="U64" s="6" t="inlineStr">
         <is>
-          <t>5750</t>
+          <t>5600</t>
         </is>
       </c>
     </row>
@@ -7751,7 +7919,7 @@
       </c>
       <c r="U65" s="6" t="inlineStr">
         <is>
-          <t>5760</t>
+          <t>5610</t>
         </is>
       </c>
     </row>
@@ -7763,7 +7931,7 @@
       </c>
       <c r="U66" s="6" t="inlineStr">
         <is>
-          <t>5770</t>
+          <t>5700</t>
         </is>
       </c>
     </row>
@@ -7775,7 +7943,7 @@
       </c>
       <c r="U67" s="6" t="inlineStr">
         <is>
-          <t>5800</t>
+          <t>5750</t>
         </is>
       </c>
     </row>
@@ -7787,7 +7955,7 @@
       </c>
       <c r="U68" s="6" t="inlineStr">
         <is>
-          <t>5900</t>
+          <t>5760</t>
         </is>
       </c>
     </row>
@@ -7799,7 +7967,7 @@
       </c>
       <c r="U69" s="6" t="inlineStr">
         <is>
-          <t>5920</t>
+          <t>5770</t>
         </is>
       </c>
     </row>
@@ -7809,6 +7977,11 @@
           <t>ET</t>
         </is>
       </c>
+      <c r="U70" s="6" t="inlineStr">
+        <is>
+          <t>5800</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="T71" s="6" t="inlineStr">
@@ -7816,6 +7989,11 @@
           <t>FI</t>
         </is>
       </c>
+      <c r="U71" s="6" t="inlineStr">
+        <is>
+          <t>5900</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="T72" s="6" t="inlineStr">
@@ -7823,11 +8001,21 @@
           <t>FJ</t>
         </is>
       </c>
+      <c r="U72" s="6" t="inlineStr">
+        <is>
+          <t>5920</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="T73" s="6" t="inlineStr">
         <is>
           <t>FK</t>
+        </is>
+      </c>
+      <c r="U73" s="6" t="inlineStr">
+        <is>
+          <t>5930</t>
         </is>
       </c>
     </row>

</xml_diff>